<commit_message>
Rename Operations Yard to Hauling Yard for consistency
Operations Yard and Hauling Yard are the same facility type and already
run the same audit form, so collapse the label to a single name. Rename
the 7 Operations Yard sites (PRR-Paramount, DART, Van Norman,
TO-Conejo Center Dr, LA South, LA North, Vincent) to Hauling Yard in the
source data, regenerate the snapshot, and rebuild the review workbook so
the Assignment Confirmation tab shows the consistent label.

TYPE_TEMPLATE keeps the Operations Yard alias mapping to the hauling form
as a harmless fallback for any older stored data.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01My8dNPfGAumBY1iDLJ9YPS
</commit_message>
<xml_diff>
--- a/docs/Athens_Audit_Checklists_for_Review.xlsx
+++ b/docs/Athens_Audit_Checklists_for_Review.xlsx
@@ -950,7 +950,7 @@
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>Operations Yard</t>
+          <t>Hauling Yard</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Operations Yard</t>
+          <t>Hauling Yard</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Operations Yard</t>
+          <t>Hauling Yard</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="C20" s="21" t="inlineStr">
         <is>
-          <t>Operations Yard</t>
+          <t>Hauling Yard</t>
         </is>
       </c>
       <c r="D20" s="22" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Operations Yard</t>
+          <t>Hauling Yard</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>Operations Yard</t>
+          <t>Hauling Yard</t>
         </is>
       </c>
       <c r="D34" s="22" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Operations Yard</t>
+          <t>Hauling Yard</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">

</xml_diff>